<commit_message>
effort: reconcile rollup with shipped work
Updates seven stale Status cells the autonomous loop forgot to flip
when it merged the corresponding PRs:

- S011 DashboardView                    → Done (M-07-DASH + UI sweep)
- B004 Admin (api/v1/admin.py)          → Done (CQR-4 split + P0-06)
- B025 Alembic migrations               → Done (P0-04)
- B026 Persistent users + admin (P0-06) → Done
- B027 Persistent eval scoring (B-08)   → Done
- B028 End-to-end smoke test (P0-07)    → Done
- M018 MediaPipe face detection         → Not Started
                                          (was misreported as In Progress;
                                          actual integration deferred to
                                          pilot follow-up — see
                                          AUR-MP-CROSSCHECK in backlog)

Formulas on the Effort Summary tab pick this up automatically when
Excel reopens the workbook.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MVP_Effort_Estimation_Aurion.xlsx
+++ b/MVP_Effort_Estimation_Aurion.xlsx
@@ -2311,7 +2311,7 @@
       </c>
       <c r="K14" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L14" s="37" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="L7" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M7" s="37" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="L28" s="37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M28" s="37" t="inlineStr">
@@ -5953,7 +5953,7 @@
       </c>
       <c r="L29" s="37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M29" s="37" t="inlineStr">
@@ -6044,7 +6044,7 @@
       </c>
       <c r="L30" s="37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M30" s="37" t="inlineStr">
@@ -6135,7 +6135,7 @@
       </c>
       <c r="L31" s="37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M31" s="37" t="inlineStr">
@@ -8241,7 +8241,7 @@
       </c>
       <c r="M21" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="N21" s="37" t="inlineStr">

</xml_diff>